<commit_message>
feat(F-AUD-006): passe corpus 1445 histoires, colonne script
Chaque chunk a un script role|phrase. Le texte enfant n’annonce
plus maman dit / papa dit.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -602,7 +602,6 @@
           <t>secondary_lessons</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -819,6 +818,18 @@
       <c r="B29" t="inlineStr">
         <is>
           <t>xlsx-arbre-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>voice_cast</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>voix-roles-v1</t>
         </is>
       </c>
     </row>
@@ -833,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV6"/>
+  <dimension ref="A1:AW6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1127,6 +1138,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1151,7 +1167,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>C'est le matin. Tom est dans l'entrée. Le sac est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte. Papa dit : la gourde, le doudou, le livre. Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac. Papa dit : merci Tom. Le sac est prêt.</t>
+          <t>C'est le matin. Tom est dans l'entrée. Le sac est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte. La gourde, le doudou, le livre. Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac. Merci Tom. Le sac est prêt.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1289,6 +1305,15 @@
         <v>12</v>
       </c>
       <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>narrateur|C'est le matin. Tom est dans l'entrée. Le sac est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte.
+papa|La gourde, le doudou, le livre.
+narrateur|Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac.
+papa|Merci Tom.
+narrateur|Le sac est prêt.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1469,6 +1494,11 @@
       <c r="AV3" s="2" t="inlineStr">
         <is>
           <t>question d'écoute, ne change pas le cours</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>narrateur|Tom prépare le sac. Que fait-il ?</t>
         </is>
       </c>
     </row>
@@ -1637,6 +1667,11 @@
           <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
         </is>
       </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>narrateur|Tom a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. Le sac est prêt.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1799,6 +1834,11 @@
         <v>12</v>
       </c>
       <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>narrateur|Tom prend le sac. La sangle est lisse. Papa ouvre la porte. Ils partent.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1961,6 +2001,11 @@
         <v>12</v>
       </c>
       <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>narrateur|L'histoire est finie.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -1979,7 +2024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1996,6 +2041,13 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>conversion structurelle, prompts de choix alignés, TTS profilé</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F-AUD-006 scripts multi-voix, sans « X dit »</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-AUD-007): colonne sons sur 1445 histoires
2237 passages avec bruit, 66550 silencieux.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW6"/>
+  <dimension ref="A1:AX6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1143,11 @@
           <t>script</t>
         </is>
       </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>sons</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1314,6 +1319,7 @@
 narrateur|Le sac est prêt.</t>
         </is>
       </c>
+      <c r="AX2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1501,6 +1507,7 @@
           <t>narrateur|Tom prépare le sac. Que fait-il ?</t>
         </is>
       </c>
+      <c r="AX3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1672,6 +1679,7 @@
           <t>narrateur|Tom a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. Le sac est prêt.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1839,6 +1847,7 @@
           <t>narrateur|Tom prend le sac. La sangle est lisse. Papa ouvre la porte. Ils partent.</t>
         </is>
       </c>
+      <c r="AX5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2006,6 +2015,7 @@
           <t>narrateur|L'histoire est finie.</t>
         </is>
       </c>
+      <c r="AX6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2024,7 +2034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2048,6 +2058,20 @@
       <c r="A3" t="inlineStr">
         <is>
           <t>F-AUD-006 scripts multi-voix, sans « X dit »</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2249,6 +2273,18 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sons</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ids de bruits (vide = silence). Le bruit se joue, puis l'histoire reprend au calme.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(F-NAR-009): nouvelle vague d’atomiques réécrites
Ouvertures descriptives, troupe D16, texte seulement.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tom prépare son sac</t>
+          <t>Le sac bleu d'Amir</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Un carré de lumière montre le sac bleu. Amir y met la gourde, le doudou et le livre. Papa dit merci. Ils partent.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>C'est le matin. Tom est dans l'entrée. Le sac est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte. La gourde, le doudou, le livre. Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac. Merci Tom. Le sac est prêt.</t>
+          <t>Un carré de lumière pose sur le tapis. Il est jaune et chaud. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. La maison sent le pain. Dehors, un oiseau fait un petit cri. Amir, viens voir. En ce moment, Amir s'accroupit. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Tu la mets dans le sac ? Amir prend la gourde. Le bouchon fait clic. Il la met dans le sac. Bravo. La gourde est dedans. Amir voit le doudou doux. Le doudou sent le lit. Il est tout doux. Tu le mets dans le sac ? Amir prend le doudou. Il le glisse dans le sac. Bravo. Le doudou est dedans. Amir voit le petit livre. La couverture est lisse. Tu mets le livre aussi ? Amir prend le livre. Il le met dans le sac. Tu as mis ce que l'adulte a dit. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Merci Amir. Le sac est prêt ? Oui, papa. Bravo. Tu as fait du bon travail. Le carré de lumière brille encore.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,14 +1324,52 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|C'est le matin. Tom est dans l'entrée. Le sac est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte.
+          <t>narrateur|Un carré de lumière pose sur le tapis.
+narrateur|Il est jaune et chaud.
+narrateur|Les chaussures de papa sentent le cuir.
+narrateur|Un manteau bleu pend au crochet.
+narrateur|La maison sent le pain.
+narrateur|Dehors, un oiseau fait un petit cri.
+papa|Amir, viens voir.
+narrateur|En ce moment, Amir s'accroupit.
+narrateur|Le sac bleu est par terre.
+narrateur|La sangle est lisse.
+enfant-m|Il est bleu, papa.
+papa|Oui. C'est ton sac.
+papa|On met ce que l'adulte a dit.
 papa|La gourde, le doudou, le livre.
-narrateur|Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac.
-papa|Merci Tom.
-narrateur|Le sac est prêt.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+enfant-m|La gourde, le doudou, le livre.
+narrateur|Amir écoute.
+narrateur|Il voit la gourde bleue.
+narrateur|Elle est un peu froide.
+papa|Tu la mets dans le sac ?
+narrateur|Amir prend la gourde.
+narrateur|Le bouchon fait clic.
+narrateur|Il la met dans le sac.
+papa|Bravo. La gourde est dedans.
+narrateur|Amir voit le doudou doux.
+narrateur|Le doudou sent le lit.
+enfant-m|Il est tout doux.
+papa|Tu le mets dans le sac ?
+narrateur|Amir prend le doudou.
+narrateur|Il le glisse dans le sac.
+papa|Bravo. Le doudou est dedans.
+narrateur|Amir voit le petit livre.
+narrateur|La couverture est lisse.
+papa|Tu mets le livre aussi ?
+narrateur|Amir prend le livre.
+narrateur|Il le met dans le sac.
+papa|Tu as mis ce que l'adulte a dit.
+narrateur|Amir appuie sur la fermeture.
+narrateur|Ça fait zzz.
+narrateur|Le sac est fermé.
+papa|Merci Amir.
+papa|Le sac est prêt ?
+enfant-m|Oui, papa.
+papa|Bravo. Tu as fait du bon travail.
+narrateur|Le carré de lumière brille encore.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1344,7 +1394,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Tom prépare le sac. Que fait-il ?</t>
+          <t>Amir prépare le sac. Que fait-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1504,10 +1554,10 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Tom prépare le sac. Que fait-il ?</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr"/>
+          <t>narrateur|Amir prépare le sac.
+narrateur|Que fait-il ?</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1532,7 +1582,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Tom a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. Le sac est prêt.</t>
+          <t>Amir a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. C'est ce que l'adulte a dit. Tu as fini de préparer le sac ? Oui. Bravo. Le sac est prêt. Amir pose la main sur le sac. Le tissu est un peu rêche. Le carré jaune reste sur le tapis.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1676,10 +1726,19 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Tom a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. Le sac est prêt.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+          <t>narrateur|Amir a écouté.
+narrateur|Il a mis la gourde.
+narrateur|Il a mis le doudou.
+narrateur|Il a mis le livre.
+narrateur|C'est ce que l'adulte a dit.
+papa|Tu as fini de préparer le sac ?
+enfant-m|Oui.
+papa|Bravo. Le sac est prêt.
+narrateur|Amir pose la main sur le sac.
+narrateur|Le tissu est un peu rêche.
+narrateur|Le carré jaune reste sur le tapis.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1704,7 +1763,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tom prend le sac. La sangle est lisse. Papa ouvre la porte. Ils partent.</t>
+          <t>Amir prend le sac. La sangle est lisse. On met tes chaussures ? Amir enfile ses chaussures. Tu as fini tes chaussures ? Oui, papa. Bravo. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Ils partent. Le sac bleu tape doucement.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1844,10 +1903,20 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Tom prend le sac. La sangle est lisse. Papa ouvre la porte. Ils partent.</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr"/>
+          <t>narrateur|Amir prend le sac.
+narrateur|La sangle est lisse.
+papa|On met tes chaussures ?
+narrateur|Amir enfile ses chaussures.
+papa|Tu as fini tes chaussures ?
+enfant-m|Oui, papa.
+papa|Bravo.
+papa|On ouvre la porte.
+narrateur|Papa ouvre la porte.
+narrateur|L'air sent le pain du village.
+narrateur|Ils partent.
+narrateur|Le sac bleu tape doucement.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1872,7 +1941,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est sur le dos d'Amir. La gourde, le doudou, le livre. Le sac est prêt. Oui. Tu as mis ce que l'adulte a dit. Bravo, Amir. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2012,10 +2081,14 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr"/>
+          <t>narrateur|Le sac est sur le dos d'Amir.
+narrateur|La gourde, le doudou, le livre.
+enfant-m|Le sac est prêt.
+papa|Oui. Tu as mis ce que l'adulte a dit.
+papa|Bravo, Amir.
+narrateur|L'histoire est finie.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2034,7 +2107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2072,6 +2145,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-009): 135 textes locaux plus récents que main
Les branches git n’avaient pas de divergence : tout était déjà dans main.
Le working tree avait des xlsx plus récents (réécritures). On les garde.
TREE-COL-007 et TREE-COL-008 locaux étaient des régressions : version main conservée.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -1184,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un carré de lumière pose sur le tapis. Il est jaune et chaud. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. La maison sent le pain. Dehors, un oiseau fait un petit cri. Amir, viens voir. En ce moment, Amir s'accroupit. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Tu la mets dans le sac ? Amir prend la gourde. Le bouchon fait clic. Il la met dans le sac. Bravo. La gourde est dedans. Amir voit le doudou doux. Le doudou sent le lit. Il est tout doux. Tu le mets dans le sac ? Amir prend le doudou. Il le glisse dans le sac. Bravo. Le doudou est dedans. Amir voit le petit livre. La couverture est lisse. Tu mets le livre aussi ? Amir prend le livre. Il le met dans le sac. Tu as mis ce que l'adulte a dit. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Merci Amir. Le sac est prêt ? Oui, papa. Bravo. Tu as fait du bon travail. Le carré de lumière brille encore.</t>
+          <t>Un carré de lumière se pose sur le tapis. Il est jaune et chaud. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. La maison sent le pain. Dehors, un oiseau fait un petit cri. Amir, viens voir. En ce moment, Amir s'accroupit. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Tu la mets dans le sac ? Amir prend la gourde. Le bouchon fait clic. Il la met dans le sac. Bravo. La gourde est dedans. Amir voit le doudou doux. Le doudou sent le lit. Il est tout doux. Tu le mets dans le sac ? Amir prend le doudou. Il le glisse dans le sac. Bravo. Le doudou est dedans. Amir voit le petit livre. La couverture est lisse. Tu mets le livre aussi ? Amir prend le livre. Il le met dans le sac. Tu as mis ce que l'adulte a dit. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Merci Amir. Le sac est prêt ? Oui, papa. Bravo. Tu as fait du bon travail. Le carré de lumière brille encore.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1324,7 +1324,7 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un carré de lumière pose sur le tapis.
+          <t>narrateur|Un carré de lumière se pose sur le tapis.
 narrateur|Il est jaune et chaud.
 narrateur|Les chaussures de papa sentent le cuir.
 narrateur|Un manteau bleu pend au crochet.
@@ -2107,7 +2107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2150,6 +2150,34 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-008): 64 ATOM, vraies histoires (vague 1)
Monde, désir, imprévu, fin. Plus des puces de leçon. Voix Piper plus lentes (bake plus tard).
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le sac bleu d'Amir</t>
+          <t>Le pain et le sac d'Amir</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>entrée de la maison</t>
+          <t>entrée puis chemin du village</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tom, papa</t>
+          <t>Amir, papa</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20">
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>150</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21">
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Un carré de lumière montre le sac bleu. Amir y met la gourde, le doudou et le livre. Papa dit merci. Ils partent.</t>
+          <t>Amir veut aller sentir le pain du village. Papa dit gourde, doudou, livre. Le doudou est encore sur le lit. Amir les met dans le sac bleu. Ils marchent. Le four est tout près.</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un carré de lumière se pose sur le tapis. Il est jaune et chaud. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. La maison sent le pain. Dehors, un oiseau fait un petit cri. Amir, viens voir. En ce moment, Amir s'accroupit. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Tu la mets dans le sac ? Amir prend la gourde. Le bouchon fait clic. Il la met dans le sac. Bravo. La gourde est dedans. Amir voit le doudou doux. Le doudou sent le lit. Il est tout doux. Tu le mets dans le sac ? Amir prend le doudou. Il le glisse dans le sac. Bravo. Le doudou est dedans. Amir voit le petit livre. La couverture est lisse. Tu mets le livre aussi ? Amir prend le livre. Il le met dans le sac. Tu as mis ce que l'adulte a dit. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Merci Amir. Le sac est prêt ? Oui, papa. Bravo. Tu as fait du bon travail. Le carré de lumière brille encore.</t>
+          <t>Le pain du village sent encore le four. L'odeur glisse sous la porte. Elle est tiède et douce. La table de la cuisine est encore chaude. Papa essuie une petite miette. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée est un peu rêche. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Le bouchon fait clic. Amir la pose dans le sac. La gourde est dedans. Oui. Maintenant le livre. Le petit livre est sur le banc. La couverture est lisse. Amir le glisse dans le sac. Où est mon doudou ? Le sac a un creux tout doux. Le doudou n'est pas là. Il attend sur le lit. Je vais le chercher.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est le matin. Tom est dans l'entrée. Le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte. Papa dit : la gourde, le doudou, le livre. Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac. Papa dit : merci Tom. Le sac est prêt.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le pain du village sent encore le four. L'odeur glisse sous la porte. Elle est tiède et douce. La table de la cuisine est encore chaude. Papa essuie une petite miette. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée est un peu rêche. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Le bouchon fait clic. Amir la pose dans le sac. La gourde est dedans. Oui. Maintenant le livre. Le petit livre est sur le banc. La couverture est lisse. Amir le glisse dans le sac. Où est mon doudou ? Le sac a un creux tout doux. Le doudou n'est pas là. Il attend sur le lit. Je vais le chercher.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
         <v>0.86</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1324,14 +1324,21 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un carré de lumière se pose sur le tapis.
-narrateur|Il est jaune et chaud.
+          <t>narrateur|Le pain du village sent encore le four.
+narrateur|L'odeur glisse sous la porte.
+narrateur|Elle est tiède et douce.
+narrateur|La table de la cuisine est encore chaude.
+narrateur|Papa essuie une petite miette.
 narrateur|Les chaussures de papa sentent le cuir.
 narrateur|Un manteau bleu pend au crochet.
-narrateur|La maison sent le pain.
+narrateur|Le tapis de l'entrée est un peu rêche.
+narrateur|Un carré de soleil touche le bois.
 narrateur|Dehors, un oiseau fait un petit cri.
-papa|Amir, viens voir.
-narrateur|En ce moment, Amir s'accroupit.
+papa|Amir, tu sens le pain ?
+enfant-m|Oui, papa.
+enfant-m|Il est chaud.
+papa|On va le voir, tout près.
+narrateur|En ce moment, Amir touche le sac.
 narrateur|Le sac bleu est par terre.
 narrateur|La sangle est lisse.
 enfant-m|Il est bleu, papa.
@@ -1342,32 +1349,18 @@
 narrateur|Amir écoute.
 narrateur|Il voit la gourde bleue.
 narrateur|Elle est un peu froide.
-papa|Tu la mets dans le sac ?
-narrateur|Amir prend la gourde.
 narrateur|Le bouchon fait clic.
-narrateur|Il la met dans le sac.
-papa|Bravo. La gourde est dedans.
-narrateur|Amir voit le doudou doux.
-narrateur|Le doudou sent le lit.
-enfant-m|Il est tout doux.
-papa|Tu le mets dans le sac ?
-narrateur|Amir prend le doudou.
-narrateur|Il le glisse dans le sac.
-papa|Bravo. Le doudou est dedans.
-narrateur|Amir voit le petit livre.
+narrateur|Amir la pose dans le sac.
+enfant-m|La gourde est dedans.
+papa|Oui. Maintenant le livre.
+narrateur|Le petit livre est sur le banc.
 narrateur|La couverture est lisse.
-papa|Tu mets le livre aussi ?
-narrateur|Amir prend le livre.
-narrateur|Il le met dans le sac.
-papa|Tu as mis ce que l'adulte a dit.
-narrateur|Amir appuie sur la fermeture.
-narrateur|Ça fait zzz.
-narrateur|Le sac est fermé.
-papa|Merci Amir.
-papa|Le sac est prêt ?
-enfant-m|Oui, papa.
-papa|Bravo. Tu as fait du bon travail.
-narrateur|Le carré de lumière brille encore.</t>
+narrateur|Amir le glisse dans le sac.
+enfant-m|Où est mon doudou ?
+narrateur|Le sac a un creux tout doux.
+narrateur|Le doudou n'est pas là.
+papa|Il attend sur le lit.
+enfant-m|Je vais le chercher.</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1387,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Amir prépare le sac. Que fait-il ?</t>
+          <t>Amir prépare le sac. Où met-il les affaires ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Tom prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Que fait-il ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir prépare le sac. Où met-il les affaires ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1414,7 +1407,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>le sac | il met | dans le sac | mettre</t>
+          <t>le sac | dans le sac | il met | mettre | la gourde | le doudou | le livre</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1429,7 +1422,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il met les affaires dans le sac. Que fait Tom ?</t>
+          <t>Il met les affaires dans le sac. Où les met-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,7 +1471,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.28</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1555,7 +1548,7 @@
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Amir prépare le sac.
-narrateur|Que fait-il ?</t>
+narrateur|Où met-il les affaires ?</t>
         </is>
       </c>
     </row>
@@ -1582,12 +1575,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. C'est ce que l'adulte a dit. Tu as fini de préparer le sac ? Oui. Bravo. Le sac est prêt. Amir pose la main sur le sac. Le tissu est un peu rêche. Le carré jaune reste sur le tapis.</t>
+          <t>Amir va vers le lit. Le doudou sent encore l'oreiller. Il est tout doux. Te voilà. Il le glisse dans le sac. Tu as mis ce que l'adulte a dit. La gourde, le doudou, le livre. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le sac. Le tissu est un peu rêche. Le creux tout doux est plein. Tu as la gourde ? Oui. Et le doudou. Et le livre aussi. Oui. Dans le sac.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Tom a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. Le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; est prêt.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir va vers le lit. Le doudou sent encore l'oreiller. Il est tout doux. Te voilà. Il le glisse dans le sac. Tu as mis ce que l'adulte a dit. La gourde, le doudou, le livre. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le sac. Le tissu est un peu rêche. Le creux tout doux est plein. Tu as la gourde ? Oui. Et le doudou. Et le livre aussi. Oui. Dans le sac.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1650,7 +1643,7 @@
         <v>0.86</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1726,17 +1719,25 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir a écouté.
-narrateur|Il a mis la gourde.
-narrateur|Il a mis le doudou.
-narrateur|Il a mis le livre.
-narrateur|C'est ce que l'adulte a dit.
-papa|Tu as fini de préparer le sac ?
-enfant-m|Oui.
-papa|Bravo. Le sac est prêt.
+          <t>narrateur|Amir va vers le lit.
+narrateur|Le doudou sent encore l'oreiller.
+narrateur|Il est tout doux.
+enfant-m|Te voilà.
+narrateur|Il le glisse dans le sac.
+papa|Tu as mis ce que l'adulte a dit.
+papa|La gourde, le doudou, le livre.
+narrateur|Amir appuie sur la fermeture.
+narrateur|Ça fait zzz.
+narrateur|Le sac est fermé.
+papa|Le sac est prêt ?
+enfant-m|Oui, papa.
 narrateur|Amir pose la main sur le sac.
 narrateur|Le tissu est un peu rêche.
-narrateur|Le carré jaune reste sur le tapis.</t>
+narrateur|Le creux tout doux est plein.
+papa|Tu as la gourde ?
+enfant-m|Oui. Et le doudou.
+papa|Et le livre aussi.
+enfant-m|Oui. Dans le sac.</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1764,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le sac. La sangle est lisse. On met tes chaussures ? Amir enfile ses chaussures. Tu as fini tes chaussures ? Oui, papa. Bravo. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Ils partent. Le sac bleu tape doucement.</t>
+          <t>On met tes chaussures. Amir enfile ses chaussures. Une semelle est un peu froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui. Il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Tom prend le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. La sangle est lisse. Papa ouvre la porte. Ils partent.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>On met tes chaussures. Amir enfile ses chaussures. Une semelle est un peu froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui. Il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1831,7 +1832,7 @@
         <v>0.86</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1903,18 +1904,22 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir prend le sac.
-narrateur|La sangle est lisse.
-papa|On met tes chaussures ?
+          <t>papa|On met tes chaussures.
 narrateur|Amir enfile ses chaussures.
+narrateur|Une semelle est un peu froide.
 papa|Tu as fini tes chaussures ?
 enfant-m|Oui, papa.
-papa|Bravo.
 papa|On ouvre la porte.
 narrateur|Papa ouvre la porte.
 narrateur|L'air sent le pain du village.
-narrateur|Ils partent.
-narrateur|Le sac bleu tape doucement.</t>
+narrateur|Le sac bleu tape doucement.
+enfant-m|On va voir le pain ?
+papa|Oui. Il est tout près.
+narrateur|Ils marchent sur le chemin.
+narrateur|Une miette de soleil reste au sol.
+narrateur|Le village sent le four, de plus en plus.
+enfant-m|Je le vois, papa ?
+papa|Bientôt. On continue.</t>
         </is>
       </c>
     </row>
@@ -1941,12 +1946,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sac est sur le dos d'Amir. La gourde, le doudou, le livre. Le sac est prêt. Oui. Tu as mis ce que l'adulte a dit. Bravo, Amir. L'histoire est finie.</t>
+          <t>Le pain sent encore plus fort. Le sac est sur le dos d'Amir. La gourde, le doudou, le livre. Oui. C'est dans le sac. Tu as mis ce que l'adulte a dit. Ils s'arrêtent devant le four tiède. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le pain sent encore plus fort. Le sac est sur le dos d'Amir. La gourde, le doudou, le livre. Oui. C'est dans le sac. Tu as mis ce que l'adulte a dit. Ils s'arrêtent devant le four tiède. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2009,7 +2014,7 @@
         <v>0.82</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.22</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2081,11 +2086,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est sur le dos d'Amir.
-narrateur|La gourde, le doudou, le livre.
-enfant-m|Le sac est prêt.
-papa|Oui. Tu as mis ce que l'adulte a dit.
-papa|Bravo, Amir.
+          <t>narrateur|Le pain sent encore plus fort.
+narrateur|Le sac est sur le dos d'Amir.
+enfant-m|La gourde, le doudou, le livre.
+papa|Oui. C'est dans le sac.
+papa|Tu as mis ce que l'adulte a dit.
+narrateur|Ils s'arrêtent devant le four tiède.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -2107,7 +2113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2180,6 +2186,13 @@
       <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-008): 55 ATOM, vraies histoires (rues, sac, cuisine)
Plus de listes de gestes. Monde, désir, imprévu, fin vécue.
AFF.001 / ROU.001 repris (plus de puces gourde-doudou-livre).
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le pain et le sac d'Amir</t>
+          <t>Le four du village</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut aller sentir le pain du village. Papa dit gourde, doudou, livre. Le doudou est encore sur le lit. Amir les met dans le sac bleu. Ils marchent. Le four est tout près.</t>
+          <t>Amir veut sentir le pain du village. Le doudou est sur le lit, la sangle coincée. Il les range dans le sac bleu. Le four lui chauffe les joues.</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le pain du village sent encore le four. L'odeur glisse sous la porte. Elle est tiède et douce. La table de la cuisine est encore chaude. Papa essuie une petite miette. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée est un peu rêche. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Le bouchon fait clic. Amir la pose dans le sac. La gourde est dedans. Oui. Maintenant le livre. Le petit livre est sur le banc. La couverture est lisse. Amir le glisse dans le sac. Où est mon doudou ? Le sac a un creux tout doux. Le doudou n'est pas là. Il attend sur le lit. Je vais le chercher.</t>
+          <t>Le four du village sent déjà le pain. L'odeur glisse sous la porte. Elle est tiède, un peu sucrée. Une miette dore encore sur la table. Papa essuie le bois du plat. Les chaussures sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée gratte un peu. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse, un peu froide. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four aussi. Où est mon doudou ? Le sac a un creux tout vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent encore le pain. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent encore l'oreiller. Te voilà. Amir le serre contre sa joue. Le tissu est chaud, tout doux. Tu l'as trouvé ? Oui. Il vient avec nous. Glisse-le dans le sac. Amir revient vers l'entrée. La sangle reste coincée sous la chaise. Ça ne veut pas, papa. Tire tout doucement.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le pain du village sent encore le four. L'odeur glisse sous la porte. Elle est tiède et douce. La table de la cuisine est encore chaude. Papa essuie une petite miette. Les chaussures de papa sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée est un peu rêche. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse. Il est bleu, papa. Oui. C'est ton sac. On met ce que l'adulte a dit. La gourde, le doudou, le livre. La gourde, le doudou, le livre. Amir écoute. Il voit la gourde bleue. Elle est un peu froide. Le bouchon fait clic. Amir la pose dans le sac. La gourde est dedans. Oui. Maintenant le livre. Le petit livre est sur le banc. La couverture est lisse. Amir le glisse dans le sac. Où est mon doudou ? Le sac a un creux tout doux. Le doudou n'est pas là. Il attend sur le lit. Je vais le chercher.</t>
+          <t>Le four du village sent déjà le pain. L'odeur glisse sous la porte. Elle est tiède, un peu sucrée. Une miette dore encore sur la table. Papa essuie le bois du plat. Les chaussures sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée gratte un peu. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse, un peu froide. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four aussi. Où est mon doudou ? Le sac a un creux tout vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent encore le pain. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent encore l'oreiller. Te voilà. Amir le serre contre sa joue. Le tissu est chaud, tout doux. Tu l'as trouvé ? Oui. Il vient avec nous. Glisse-le dans le sac. Amir revient vers l'entrée. La sangle reste coincée sous la chaise. Ça ne veut pas, papa. Tire tout doucement.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
@@ -1324,14 +1324,14 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le pain du village sent encore le four.
+          <t>narrateur|Le four du village sent déjà le pain.
 narrateur|L'odeur glisse sous la porte.
-narrateur|Elle est tiède et douce.
-narrateur|La table de la cuisine est encore chaude.
-narrateur|Papa essuie une petite miette.
-narrateur|Les chaussures de papa sentent le cuir.
+narrateur|Elle est tiède, un peu sucrée.
+narrateur|Une miette dore encore sur la table.
+narrateur|Papa essuie le bois du plat.
+narrateur|Les chaussures sentent le cuir.
 narrateur|Un manteau bleu pend au crochet.
-narrateur|Le tapis de l'entrée est un peu rêche.
+narrateur|Le tapis de l'entrée gratte un peu.
 narrateur|Un carré de soleil touche le bois.
 narrateur|Dehors, un oiseau fait un petit cri.
 papa|Amir, tu sens le pain ?
@@ -1340,27 +1340,38 @@
 papa|On va le voir, tout près.
 narrateur|En ce moment, Amir touche le sac.
 narrateur|Le sac bleu est par terre.
-narrateur|La sangle est lisse.
+narrateur|La sangle est lisse, un peu froide.
 enfant-m|Il est bleu, papa.
-papa|Oui. C'est ton sac.
-papa|On met ce que l'adulte a dit.
-papa|La gourde, le doudou, le livre.
-enfant-m|La gourde, le doudou, le livre.
-narrateur|Amir écoute.
-narrateur|Il voit la gourde bleue.
-narrateur|Elle est un peu froide.
-narrateur|Le bouchon fait clic.
-narrateur|Amir la pose dans le sac.
-enfant-m|La gourde est dedans.
-papa|Oui. Maintenant le livre.
-narrateur|Le petit livre est sur le banc.
-narrateur|La couverture est lisse.
-narrateur|Amir le glisse dans le sac.
+papa|Oui, c'est le tien.
+papa|Prends de l'eau, pour le chemin.
+narrateur|Amir prend la gourde bleue.
+narrateur|Le bouchon est froid sous le doigt.
+narrateur|Il fait clic, tout petit.
+narrateur|Amir pose la gourde dans le sac.
+enfant-m|Elle est un peu froide.
+papa|Elle se réchauffera dehors.
+papa|Ton doudou voudra le four aussi.
 enfant-m|Où est mon doudou ?
-narrateur|Le sac a un creux tout doux.
+narrateur|Le sac a un creux tout vide.
 narrateur|Le doudou n'est pas là.
-papa|Il attend sur le lit.
-enfant-m|Je vais le chercher.</t>
+papa|Il attend sur le lit ?
+enfant-m|Je vais le chercher.
+narrateur|Amir part vers la chambre.
+narrateur|Le couloir sent encore le pain.
+narrateur|Le plancher est un peu froid.
+narrateur|Sur le lit, le doudou attend.
+narrateur|Il sent encore l'oreiller.
+enfant-m|Te voilà.
+narrateur|Amir le serre contre sa joue.
+narrateur|Le tissu est chaud, tout doux.
+papa|Tu l'as trouvé ?
+enfant-m|Oui.
+enfant-m|Il vient avec nous.
+papa|Glisse-le dans le sac.
+narrateur|Amir revient vers l'entrée.
+narrateur|La sangle reste coincée sous la chaise.
+enfant-m|Ça ne veut pas, papa.
+papa|Tire tout doucement.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1418,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>le sac | dans le sac | il met | mettre | la gourde | le doudou | le livre</t>
+          <t>le sac | dans le sac | il met | elle met | mettre</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1422,7 +1433,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il met les affaires dans le sac. Où les met-il ?</t>
+          <t>Il met les affaires dans le sac. Où les met Amir ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1575,12 +1586,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir va vers le lit. Le doudou sent encore l'oreiller. Il est tout doux. Te voilà. Il le glisse dans le sac. Tu as mis ce que l'adulte a dit. La gourde, le doudou, le livre. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le sac. Le tissu est un peu rêche. Le creux tout doux est plein. Tu as la gourde ? Oui. Et le doudou. Et le livre aussi. Oui. Dans le sac.</t>
+          <t>Amir tire la sangle, tout doux. La chaise bouge un tout petit peu. La sangle se libère, lisse encore. Elle est libre. Merci, Amir. Il glisse le doudou dans le sac. Le creux n'est plus vide. Prends aussi le petit livre. Le livre est sur le banc. La couverture est lisse, un peu froide. Amir le pose près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait zzz, tout bas. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche. Le creux tout doux est plein.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir va vers le lit. Le doudou sent encore l'oreiller. Il est tout doux. Te voilà. Il le glisse dans le sac. Tu as mis ce que l'adulte a dit. La gourde, le doudou, le livre. Amir appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le sac. Le tissu est un peu rêche. Le creux tout doux est plein. Tu as la gourde ? Oui. Et le doudou. Et le livre aussi. Oui. Dans le sac.</t>
+          <t>Amir tire la sangle, tout doux. La chaise bouge un tout petit peu. La sangle se libère, lisse encore. Elle est libre. Merci, Amir. Il glisse le doudou dans le sac. Le creux n'est plus vide. Prends aussi le petit livre. Le livre est sur le banc. La couverture est lisse, un peu froide. Amir le pose près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait zzz, tout bas. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche. Le creux tout doux est plein.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1636,7 +1647,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
@@ -1719,25 +1730,27 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir va vers le lit.
-narrateur|Le doudou sent encore l'oreiller.
-narrateur|Il est tout doux.
-enfant-m|Te voilà.
-narrateur|Il le glisse dans le sac.
-papa|Tu as mis ce que l'adulte a dit.
-papa|La gourde, le doudou, le livre.
+          <t>narrateur|Amir tire la sangle, tout doux.
+narrateur|La chaise bouge un tout petit peu.
+narrateur|La sangle se libère, lisse encore.
+enfant-m|Elle est libre.
+papa|Merci, Amir.
+narrateur|Il glisse le doudou dans le sac.
+narrateur|Le creux n'est plus vide.
+papa|Prends aussi le petit livre.
+narrateur|Le livre est sur le banc.
+narrateur|La couverture est lisse, un peu froide.
+narrateur|Amir le pose près de l'eau.
+enfant-m|Il est dedans.
+papa|Tu fermes, maintenant ?
 narrateur|Amir appuie sur la fermeture.
-narrateur|Ça fait zzz.
-narrateur|Le sac est fermé.
+narrateur|Ça fait zzz, tout bas.
+narrateur|Le sac bleu est fermé.
 papa|Le sac est prêt ?
 enfant-m|Oui, papa.
-narrateur|Amir pose la main sur le sac.
+narrateur|Amir pose la main sur le tissu.
 narrateur|Le tissu est un peu rêche.
-narrateur|Le creux tout doux est plein.
-papa|Tu as la gourde ?
-enfant-m|Oui. Et le doudou.
-papa|Et le livre aussi.
-enfant-m|Oui. Dans le sac.</t>
+narrateur|Le creux tout doux est plein.</t>
         </is>
       </c>
     </row>
@@ -1764,12 +1777,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures. Amir enfile ses chaussures. Une semelle est un peu froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui. Il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue.</t>
+          <t>On met tes chaussures ? Amir enfile ses chaussures. Une semelle est encore froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue. Une poule traverse tout loin. Le chemin est un peu poudreux. Amir sent le pain sur sa langue. Ça sent bon. Oui, très bon.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures. Amir enfile ses chaussures. Une semelle est un peu froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui. Il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue.</t>
+          <t>On met tes chaussures ? Amir enfile ses chaussures. Une semelle est encore froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue. Une poule traverse tout loin. Le chemin est un peu poudreux. Amir sent le pain sur sa langue. Ça sent bon. Oui, très bon.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1825,7 +1838,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
@@ -1904,9 +1917,9 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On met tes chaussures.
+          <t>papa|On met tes chaussures ?
 narrateur|Amir enfile ses chaussures.
-narrateur|Une semelle est un peu froide.
+narrateur|Une semelle est encore froide.
 papa|Tu as fini tes chaussures ?
 enfant-m|Oui, papa.
 papa|On ouvre la porte.
@@ -1914,12 +1927,18 @@
 narrateur|L'air sent le pain du village.
 narrateur|Le sac bleu tape doucement.
 enfant-m|On va voir le pain ?
-papa|Oui. Il est tout près.
+papa|Oui, il est tout près.
 narrateur|Ils marchent sur le chemin.
 narrateur|Une miette de soleil reste au sol.
 narrateur|Le village sent le four, de plus en plus.
 enfant-m|Je le vois, papa ?
-papa|Bientôt. On continue.</t>
+papa|Bientôt.
+papa|On continue.
+narrateur|Une poule traverse tout loin.
+narrateur|Le chemin est un peu poudreux.
+narrateur|Amir sent le pain sur sa langue.
+enfant-m|Ça sent bon.
+papa|Oui, très bon.</t>
         </is>
       </c>
     </row>
@@ -1946,12 +1965,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore plus fort. Le sac est sur le dos d'Amir. La gourde, le doudou, le livre. Oui. C'est dans le sac. Tu as mis ce que l'adulte a dit. Ils s'arrêtent devant le four tiède. L'histoire est finie.</t>
+          <t>Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Le sac repose contre sa hanche. Le doudou sent le four, lui aussi. Tu as bien préparé le chemin. On le sent, papa. Le four tiède réchauffe encore ses joues.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le pain sent encore plus fort. Le sac est sur le dos d'Amir. La gourde, le doudou, le livre. Oui. C'est dans le sac. Tu as mis ce que l'adulte a dit. Ils s'arrêtent devant le four tiède. L'histoire est finie.</t>
+          <t>Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Le sac repose contre sa hanche. Le doudou sent le four, lui aussi. Tu as bien préparé le chemin. On le sent, papa. Le four tiède réchauffe encore ses joues.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2007,7 +2026,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
@@ -2086,13 +2105,15 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le pain sent encore plus fort.
-narrateur|Le sac est sur le dos d'Amir.
-enfant-m|La gourde, le doudou, le livre.
-papa|Oui. C'est dans le sac.
-papa|Tu as mis ce que l'adulte a dit.
-narrateur|Ils s'arrêtent devant le four tiède.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Ils s'arrêtent devant le four tiède.
+narrateur|La chaleur touche les joues d'Amir.
+enfant-m|Le pain est là.
+papa|Oui, tout chaud.
+narrateur|Le sac repose contre sa hanche.
+narrateur|Le doudou sent le four, lui aussi.
+papa|Tu as bien préparé le chemin.
+enfant-m|On le sent, papa.
+narrateur|Le four tiède réchauffe encore ses joues.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2191,6 +2212,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-01 Le four du village
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison du village puis chemin du four</t>
+          <t>cuisine au rebord, chemin poudreux, four du village</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut sentir le pain du village. Le doudou est sur le lit, la sangle coincée. Il les range dans le sac bleu. Le four lui chauffe les joues.</t>
+          <t>Un souffle chaud passe entre les volets. Sur le rebord, un grain de miette brille. Amir veut le pain du four, maintenant, dans son sac. Il tire trop fort : la sangle reste coincée. Il refuse de foncer, prépare le sac, contourne une pierre. Au four, le grain de miette dore sur le pain qu'il porte.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le four du village sent déjà le pain. L'odeur glisse sous la porte. Elle est tiède, un peu sucrée. Une miette dore encore sur la table. Papa essuie le bois du plat. Les chaussures sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée gratte un peu. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse, un peu froide. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four aussi. Où est mon doudou ? Le sac a un creux tout vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent encore le pain. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent encore l'oreiller. Te voilà. Amir le serre contre sa joue. Le tissu est chaud, tout doux. Tu l'as trouvé ? Oui. Il vient avec nous. Glisse-le dans le sac. Amir revient vers l'entrée. La sangle reste coincée sous la chaise. Ça ne veut pas, papa. Tire tout doucement.</t>
+          <t>La porte du four claque, au bout de la rue. Un souffle chaud passe entre les volets. Amir lève le nez, dans la cuisine. Sur le rebord, un grain de miette brille. Il est tout petit, papa. C'est un reste du pain d'hier. Le grain dore comme un bout de soleil. La nappe sent le bois et la farine. Un carré de soleil touche le bois. Amir, tu sens le pain ? Oui, papa. Je le veux chaud, maintenant. Le four est tout près, au village. Le sac bleu attend près de la porte. En ce moment, Amir saisit le sac. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four, lui aussi. Où est mon doudou ? Le sac a un creux vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent le four, tiède. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent l'oreiller, chaud. Te voilà. Amir le serre contre sa joue. Le tissu est chaud sous sa joue. Tu l'as trouvé ? Oui. Il vient avec nous. Amir revient vers la porte. Allez, on y va ! Il tire le sac, d'un coup. La sangle glisse sous la chaise. La chaise penche. Le sac reste coincé. Ça ne veut pas, papa. Amir ferme la bouche. Ses épaules tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes la sangle ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le four du village sent déjà le pain. L'odeur glisse sous la porte. Elle est tiède, un peu sucrée. Une miette dore encore sur la table. Papa essuie le bois du plat. Les chaussures sentent le cuir. Un manteau bleu pend au crochet. Le tapis de l'entrée gratte un peu. Un carré de soleil touche le bois. Dehors, un oiseau fait un petit cri. Amir, tu sens le pain ? Oui, papa. Il est chaud. On va le voir, tout près. En ce moment, Amir touche le sac. Le sac bleu est par terre. La sangle est lisse, un peu froide. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four aussi. Où est mon doudou ? Le sac a un creux tout vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent encore le pain. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent encore l'oreiller. Te voilà. Amir le serre contre sa joue. Le tissu est chaud, tout doux. Tu l'as trouvé ? Oui. Il vient avec nous. Glisse-le dans le sac. Amir revient vers l'entrée. La sangle reste coincée sous la chaise. Ça ne veut pas, papa. Tire tout doucement.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La porte du four claque, au bout de la rue. Un souffle chaud passe entre les volets. Amir lève le nez, dans la cuisine. Sur le rebord, un &lt;emphasis level="moderate"&gt;grain de miette&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un reste du pain d'hier. Le grain dore comme un bout de soleil. La nappe sent le bois et la farine. Un carré de soleil touche le bois. Amir, tu sens le pain ? Oui, papa. Je le veux chaud, maintenant. Le four est tout près, au village. Le sac bleu attend près de la porte. En ce moment, Amir saisit le sac. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four, lui aussi. Où est mon doudou ? Le sac a un creux vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent le four, tiède. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent l'oreiller, chaud. Te voilà. Amir le serre contre sa joue. Le tissu est chaud sous sa joue. Tu l'as trouvé ? Oui. Il vient avec nous. Amir revient vers la porte. Allez, on y va ! Il tire le sac, d'un coup. La sangle glisse sous la chaise. La chaise penche. Le sac reste coincé. Ça ne veut pas, papa. Amir ferme la bouche. Ses épaules tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes la sangle ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est le matin. Tom est dans l'entrée. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est par terre. Il est bleu. Papa est là, près de Tom. Papa est l'adulte. Papa dit : la gourde, le doudou, le livre. Tom écoute. Tom voit la gourde bleue. Il la prend. Il la met dans le sac. Tom voit le doudou doux. Il le prend. Il le met dans le sac. Tom voit le petit livre. Il le prend. Il le met dans le sac. Tom appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Tom a mis ce que l'adulte a dit. Papa pose la main sur le sac. Papa dit : merci Tom. Le sac est prêt.&lt;/slow&gt; [pause]</t>
+          <t>La porte du four claque, au bout de la rue. Un souffle chaud passe entre les volets. Amir lève le nez, dans la cuisine. Sur le rebord, un &lt;emphasis&gt;grain de miette&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un reste du pain d'hier. Le grain dore comme un bout de soleil. La nappe sent le bois et la farine. Un carré de soleil touche le bois. Amir, tu sens le pain ? Oui, papa. Je le veux chaud, maintenant. Le four est tout près, au village. Le sac bleu attend près de la porte. En ce moment, Amir saisit le sac. Il est bleu, papa. Oui, c'est le tien. Prends de l'eau, pour le chemin. Amir prend la gourde bleue. Le bouchon est froid sous le doigt. Il fait clic, tout petit. Amir pose la gourde dans le sac. Elle est un peu froide. Elle se réchauffera dehors. Ton doudou voudra le four, lui aussi. Où est mon doudou ? Le sac a un creux vide. Le doudou n'est pas là. Il attend sur le lit ? Je vais le chercher. Amir part vers la chambre. Le couloir sent le four, tiède. Le plancher est un peu froid. Sur le lit, le doudou attend. Il sent l'oreiller, chaud. Te voilà. Amir le serre contre sa joue. Le tissu est chaud sous sa joue. Tu l'as trouvé ? Oui. Il vient avec nous. Amir revient vers la porte. Allez, on y va ! Il tire le sac, d'un coup. La sangle glisse sous la chaise. La chaise penche. Le sac reste coincé. Ça ne veut pas, papa. Amir ferme la bouche. Ses épaules tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes la sangle ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>grain de miette</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,28 +1319,30 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous-texte=il_veut_le_pain_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le four du village sent déjà le pain.
-narrateur|L'odeur glisse sous la porte.
-narrateur|Elle est tiède, un peu sucrée.
-narrateur|Une miette dore encore sur la table.
-narrateur|Papa essuie le bois du plat.
-narrateur|Les chaussures sentent le cuir.
-narrateur|Un manteau bleu pend au crochet.
-narrateur|Le tapis de l'entrée gratte un peu.
+          <t>narrateur|La porte du four claque, au bout de la rue.
+narrateur|Un souffle chaud passe entre les volets.
+narrateur|Amir lève le nez, dans la cuisine.
+narrateur|Sur le rebord, un grain de miette brille.
+enfant-m|Il est tout petit, papa.
+papa|C'est un reste du pain d'hier.
+narrateur|Le grain dore comme un bout de soleil.
+narrateur|La nappe sent le bois et la farine.
 narrateur|Un carré de soleil touche le bois.
-narrateur|Dehors, un oiseau fait un petit cri.
 papa|Amir, tu sens le pain ?
 enfant-m|Oui, papa.
-enfant-m|Il est chaud.
-papa|On va le voir, tout près.
-narrateur|En ce moment, Amir touche le sac.
-narrateur|Le sac bleu est par terre.
-narrateur|La sangle est lisse, un peu froide.
+enfant-m|Je le veux chaud, maintenant.
+papa|Le four est tout près, au village.
+narrateur|Le sac bleu attend près de la porte.
+narrateur|En ce moment, Amir saisit le sac.
 enfant-m|Il est bleu, papa.
 papa|Oui, c'est le tien.
 papa|Prends de l'eau, pour le chemin.
@@ -1350,28 +1352,40 @@
 narrateur|Amir pose la gourde dans le sac.
 enfant-m|Elle est un peu froide.
 papa|Elle se réchauffera dehors.
-papa|Ton doudou voudra le four aussi.
+papa|Ton doudou voudra le four, lui aussi.
 enfant-m|Où est mon doudou ?
-narrateur|Le sac a un creux tout vide.
+narrateur|Le sac a un creux vide.
 narrateur|Le doudou n'est pas là.
 papa|Il attend sur le lit ?
 enfant-m|Je vais le chercher.
 narrateur|Amir part vers la chambre.
-narrateur|Le couloir sent encore le pain.
+narrateur|Le couloir sent le four, tiède.
 narrateur|Le plancher est un peu froid.
 narrateur|Sur le lit, le doudou attend.
-narrateur|Il sent encore l'oreiller.
+narrateur|Il sent l'oreiller, chaud.
 enfant-m|Te voilà.
 narrateur|Amir le serre contre sa joue.
-narrateur|Le tissu est chaud, tout doux.
+narrateur|Le tissu est chaud sous sa joue.
 papa|Tu l'as trouvé ?
 enfant-m|Oui.
 enfant-m|Il vient avec nous.
-papa|Glisse-le dans le sac.
-narrateur|Amir revient vers l'entrée.
-narrateur|La sangle reste coincée sous la chaise.
+narrateur|Amir revient vers la porte.
+enfant-m|Allez, on y va !
+narrateur|Il tire le sac, d'un coup.
+narrateur|La sangle glisse sous la chaise.
+narrateur|La chaise penche.
+narrateur|Le sac reste coincé.
 enfant-m|Ça ne veut pas, papa.
-papa|Tire tout doucement.</t>
+narrateur|Amir ferme la bouche.
+narrateur|Ses épaules tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes la sangle ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>volets,sac</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1417,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir prépare le sac. Où met-il les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1471,7 +1485,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1479,10 +1493,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,11 +1511,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1512,23 +1526,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1537,13 +1551,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1553,7 +1567,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous-texte=le_sac_tient_les_affaires; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1586,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir tire la sangle, tout doux. La chaise bouge un tout petit peu. La sangle se libère, lisse encore. Elle est libre. Merci, Amir. Il glisse le doudou dans le sac. Le creux n'est plus vide. Prends aussi le petit livre. Le livre est sur le banc. La couverture est lisse, un peu froide. Amir le pose près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait zzz, tout bas. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche. Le creux tout doux est plein.</t>
+          <t>Amir refuse de tirer plus fort. Il pose un genou au sol. La sangle est plate, sous le bois. Je la sors tout seul. Il pousse la chaise, un peu. La sangle se libère, lisse. Elle est libre. Merci, Amir. Il glisse le doudou dans le sac. Le creux n'est plus vide. Le livre attend sur le banc. Le livre aussi. La couverture est lisse, un peu froide. Amir veut tout mettre d'un coup. Le livre tombe contre la sangle. Oh. Il ne reprend pas trop vite. Il écoute le sac, un instant. Il pose le livre près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir tire la sangle, tout doux. La chaise bouge un tout petit peu. La sangle se libère, lisse encore. Elle est libre. Merci, Amir. Il glisse le doudou dans le sac. Le creux n'est plus vide. Prends aussi le petit livre. Le livre est sur le banc. La couverture est lisse, un peu froide. Amir le pose près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait zzz, tout bas. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche. Le creux tout doux est plein.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir refuse de tirer plus fort. Il pose un genou au sol. La sangle est plate, sous le bois. Je la sors tout seul. Il pousse la chaise, un peu. La sangle se libère, lisse. Elle est libre. Merci, Amir. Il glisse le doudou dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Le creux n'est plus vide. Le livre attend sur le banc. Le livre aussi. La couverture est lisse, un peu froide. Amir veut tout mettre d'un coup. Le livre tombe contre la sangle. Oh. Il ne reprend pas trop vite. Il écoute le sac, un instant. Il pose le livre près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom a écouté. Il a mis la gourde. Il a mis le doudou. Il a mis le livre. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est prêt.&lt;/slow&gt; [pause]</t>
+          <t>Amir refuse de tirer plus fort. Il pose un genou au sol. La sangle est plate, sous le bois. Je la sors tout seul. Il pousse la chaise, un peu. La sangle se libère, lisse. Elle est libre. Merci, Amir. Il glisse le doudou dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Le creux n'est plus vide. Le livre attend sur le banc. Le livre aussi. La couverture est lisse, un peu froide. Amir veut tout mettre d'un coup. Le livre tombe contre la sangle. Oh. Il ne reprend pas trop vite. Il écoute le sac, un instant. Il pose le livre près de l'eau. Il est dedans. Tu fermes, maintenant ? Amir appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. Le sac est prêt ? Oui, papa. Amir pose la main sur le tissu. Le tissu est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,7 +1657,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1651,10 +1665,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1684,23 +1698,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1723,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,36 +1735,48 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous-texte=il_prépare_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir tire la sangle, tout doux.
-narrateur|La chaise bouge un tout petit peu.
-narrateur|La sangle se libère, lisse encore.
+          <t>narrateur|Amir refuse de tirer plus fort.
+narrateur|Il pose un genou au sol.
+narrateur|La sangle est plate, sous le bois.
+enfant-m|Je la sors tout seul.
+narrateur|Il pousse la chaise, un peu.
+narrateur|La sangle se libère, lisse.
 enfant-m|Elle est libre.
 papa|Merci, Amir.
 narrateur|Il glisse le doudou dans le sac.
 narrateur|Le creux n'est plus vide.
-papa|Prends aussi le petit livre.
-narrateur|Le livre est sur le banc.
+narrateur|Le livre attend sur le banc.
+enfant-m|Le livre aussi.
 narrateur|La couverture est lisse, un peu froide.
-narrateur|Amir le pose près de l'eau.
+narrateur|Amir veut tout mettre d'un coup.
+narrateur|Le livre tombe contre la sangle.
+enfant-m|Oh.
+narrateur|Il ne reprend pas trop vite.
+narrateur|Il écoute le sac, un instant.
+narrateur|Il pose le livre près de l'eau.
 enfant-m|Il est dedans.
 papa|Tu fermes, maintenant ?
 narrateur|Amir appuie sur la fermeture.
-narrateur|Ça fait zzz, tout bas.
+narrateur|Ça fait un petit zzz.
 narrateur|Le sac bleu est fermé.
 papa|Le sac est prêt ?
 enfant-m|Oui, papa.
 narrateur|Amir pose la main sur le tissu.
-narrateur|Le tissu est un peu rêche.
-narrateur|Le creux tout doux est plein.</t>
+narrateur|Le tissu est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>sac,fermeture</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1803,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures ? Amir enfile ses chaussures. Une semelle est encore froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue. Une poule traverse tout loin. Le chemin est un peu poudreux. Amir sent le pain sur sa langue. Ça sent bon. Oui, très bon.</t>
+          <t>On met tes chaussures ? Amir enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape contre sa hanche. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Le village sent le four, chaud. Je le vois, papa ? Bientôt. On continue. Une poule traverse, plus loin. Le chemin est un peu poudreux. Une pierre ronde bloque le pas. Je saute par-dessus ! Amir recule d'un pas. Il refuse de foncer. Il contourne la pierre, lentement. Le sac reste bien fermé. Ça sent bon. Oui, très bon. Amir sent le pain sur sa langue.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures ? Amir enfile ses chaussures. Une semelle est encore froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pain du village. Le sac bleu tape doucement. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Une miette de soleil reste au sol. Le village sent le four, de plus en plus. Je le vois, papa ? Bientôt. On continue. Une poule traverse tout loin. Le chemin est un peu poudreux. Amir sent le pain sur sa langue. Ça sent bon. Oui, très bon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On met tes chaussures ? Amir enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le &lt;emphasis level="moderate"&gt;pain&lt;/emphasis&gt; du village. Le sac bleu tape contre sa hanche. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Le village sent le four, chaud. Je le vois, papa ? Bientôt. On continue. Une poule traverse, plus loin. Le chemin est un peu poudreux. Une pierre ronde bloque le pas. Je saute par-dessus ! Amir recule d'un pas. Il refuse de foncer. Il contourne la pierre, lentement. Le sac reste bien fermé. Ça sent bon. Oui, très bon. Amir sent le pain sur sa langue.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom prend le &lt;emphasis&gt;sac&lt;/emphasis&gt;. La sangle est lisse. Papa ouvre la porte. Ils partent.&lt;/slow&gt; [pause]</t>
+          <t>On met tes chaussures ? Amir enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le &lt;emphasis&gt;pain&lt;/emphasis&gt; du village. Le sac bleu tape contre sa hanche. On va voir le pain ? Oui, il est tout près. Ils marchent sur le chemin. Le village sent le four, chaud. Je le vois, papa ? Bientôt. On continue. Une poule traverse, plus loin. Le chemin est un peu poudreux. Une pierre ronde bloque le pas. Je saute par-dessus ! Amir recule d'un pas. Il refuse de foncer. Il contourne la pierre, lentement. Le sac reste bien fermé. Ça sent bon. Oui, très bon. Amir sent le pain sur sa langue. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1860,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,10 +1868,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1868,30 +1894,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>pain</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1926,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1912,33 +1938,47 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous-texte=il_refuse_de_sauter_la_pierre; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>papa|On met tes chaussures ?
 narrateur|Amir enfile ses chaussures.
-narrateur|Une semelle est encore froide.
+narrateur|Une semelle est froide.
 papa|Tu as fini tes chaussures ?
 enfant-m|Oui, papa.
 papa|On ouvre la porte.
 narrateur|Papa ouvre la porte.
 narrateur|L'air sent le pain du village.
-narrateur|Le sac bleu tape doucement.
+narrateur|Le sac bleu tape contre sa hanche.
 enfant-m|On va voir le pain ?
 papa|Oui, il est tout près.
 narrateur|Ils marchent sur le chemin.
-narrateur|Une miette de soleil reste au sol.
-narrateur|Le village sent le four, de plus en plus.
+narrateur|Le village sent le four, chaud.
 enfant-m|Je le vois, papa ?
 papa|Bientôt.
 papa|On continue.
-narrateur|Une poule traverse tout loin.
+narrateur|Une poule traverse, plus loin.
 narrateur|Le chemin est un peu poudreux.
-narrateur|Amir sent le pain sur sa langue.
+narrateur|Une pierre ronde bloque le pas.
+enfant-m|Je saute par-dessus !
+narrateur|Amir recule d'un pas.
+narrateur|Il refuse de foncer.
+narrateur|Il contourne la pierre, lentement.
+narrateur|Le sac reste bien fermé.
 enfant-m|Ça sent bon.
-papa|Oui, très bon.</t>
+papa|Oui, très bon.
+narrateur|Amir sent le pain sur sa langue.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>chemin,pas</t>
         </is>
       </c>
     </row>
@@ -1965,17 +2005,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Le sac repose contre sa hanche. Le doudou sent le four, lui aussi. Tu as bien préparé le chemin. On le sent, papa. Le four tiède réchauffe encore ses joues.</t>
+          <t>Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Un pain rond attend sur la planche. Sur la croûte, un grain de miette brille. Comme sur le rebord, papa ! Tu le portes, toi ? Oui, dans mon sac. Amir ouvre le sac, sans se presser. Il glisse le pain contre le doudou. Le sac repose contre sa hanche. On le sent, papa. Tu le sens sur tes joues ? Oui, il est chaud. Le four tiède touche ses joues. Le grain de miette dore sur le pain.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Le sac repose contre sa hanche. Le doudou sent le four, lui aussi. Tu as bien préparé le chemin. On le sent, papa. Le four tiède réchauffe encore ses joues.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Un pain rond attend sur la planche. Sur la croûte, un &lt;emphasis level="moderate"&gt;grain de miette&lt;/emphasis&gt; brille. Comme sur le rebord, papa ! Tu le portes, toi ? Oui, dans mon sac. Amir ouvre le sac, sans se presser. Il glisse le pain contre le doudou. Le sac repose contre sa hanche. On le sent, papa. Tu le sens sur tes joues ? Oui, il est chaud. Le four tiède touche ses joues. Le grain de miette dore sur le pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent devant le four tiède. La chaleur touche les joues d'Amir. Le pain est là. Oui, tout chaud. Un pain rond attend sur la planche. Sur la croûte, un &lt;emphasis&gt;grain de miette&lt;/emphasis&gt; brille. Comme sur le rebord, papa ! Tu le portes, toi ? Oui, dans mon sac. Amir ouvre le sac, sans se presser. Il glisse le pain contre le doudou. Le sac repose contre sa hanche. On le sent, papa. Tu le sens sur tes joues ? Oui, il est chaud. Le four tiède touche ses joues. Le grain de miette dore sur le pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,18 +2062,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2082,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,17 +2096,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>grain de miette</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2075,11 +2119,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,32 +2132,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous-texte=le_grain_du_rebord_est_sur_le_pain; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Ils s'arrêtent devant le four tiède.
 narrateur|La chaleur touche les joues d'Amir.
 enfant-m|Le pain est là.
 papa|Oui, tout chaud.
+narrateur|Un pain rond attend sur la planche.
+narrateur|Sur la croûte, un grain de miette brille.
+enfant-m|Comme sur le rebord, papa !
+papa|Tu le portes, toi ?
+enfant-m|Oui, dans mon sac.
+narrateur|Amir ouvre le sac, sans se presser.
+narrateur|Il glisse le pain contre le doudou.
 narrateur|Le sac repose contre sa hanche.
-narrateur|Le doudou sent le four, lui aussi.
-papa|Tu as bien préparé le chemin.
 enfant-m|On le sent, papa.
-narrateur|Le four tiède réchauffe encore ses joues.</t>
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, il est chaud.
+narrateur|Le four tiède touche ses joues.
+narrateur|Le grain de miette dore sur le pain.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>four,pain</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2219,6 +2280,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>